<commit_message>
Alevia: o singura pozitie pentru fiecare ambalaj fizic
Flacoanele sunt grupate dupa marimea etichetei (7 pozitii in loc de 21),
iar la produsele in cutie este trecut ambalajul interior (flacon, plic,
blister sau punga), cu mentiune de confirmat unde nu se vede.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VN6aeEAMfjPq2ybogLFkeD
</commit_message>
<xml_diff>
--- a/Alevia/MIRALEDO_Analiza_Ambalaje_ALEVIA.xlsx
+++ b/Alevia/MIRALEDO_Analiza_Ambalaje_ALEVIA.xlsx
@@ -1956,7 +1956,7 @@
       </c>
       <c r="C21" s="130" t="inlineStr">
         <is>
-          <t>365 produse pe alevia.ro (28.10.2026); 46 unitati de ambalaj identificate pana acum</t>
+          <t>365 produse pe alevia.ro (28.10.2026); 40 unitati de ambalaj identificate pana acum</t>
         </is>
       </c>
       <c r="D21" s="131" t="n"/>
@@ -2080,7 +2080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N60"/>
+  <dimension ref="B2:N54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" style="128" min="1" max="1"/>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="C7" s="133" t="inlineStr">
         <is>
-          <t>Blister(e) 30 comprimate masticabile (in cutie)</t>
+          <t>Blister comprimate masticabile (in cutie)</t>
         </is>
       </c>
       <c r="D7" s="133" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="F7" s="133" t="inlineStr">
         <is>
-          <t>Vitamina C cu pulpă de măceșe cu stevie Blister 30 comprimate masticabile</t>
+          <t>Propolis Vitamina C cu Echinacea Blister 20 comprimate masticabile; Vitamina C cu pulpă de măceșe cu stevie Blister 30 comprimate masticabile</t>
         </is>
       </c>
       <c r="G7" s="132" t="n"/>
@@ -2227,7 +2227,7 @@
       </c>
       <c r="C8" s="133" t="inlineStr">
         <is>
-          <t>Blister(e) 20 comprimate (in cutie)</t>
+          <t>Blister comprimate (in cutie)</t>
         </is>
       </c>
       <c r="D8" s="133" t="inlineStr">
@@ -2242,7 +2242,7 @@
       </c>
       <c r="F8" s="133" t="inlineStr">
         <is>
-          <t>Silfide Complex de slăbit forte Blister 20 comprimate</t>
+          <t>Montant Manșon 10 comprimate; Silfide Complex de slăbit forte Blister 20 comprimate</t>
         </is>
       </c>
       <c r="G8" s="132" t="n"/>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="C9" s="133" t="inlineStr">
         <is>
-          <t>Blister(e) 20 comprimate masticabile (in cutie)</t>
+          <t>Ambalaj interior capsule moi in cutie (blister sau flacon, de confirmat)</t>
         </is>
       </c>
       <c r="D9" s="133" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="F9" s="133" t="inlineStr">
         <is>
-          <t>Propolis Vitamina C cu Echinacea Blister 20 comprimate masticabile</t>
+          <t>Lecitina 1200mg 30 capsule moi; Omega 3 6 9 40 capsule moi; Omega 3 Forte 30 capsule moi; Silymarin Milk thistle 1000mg 30 capsule moi; Ulei de pește Omega 3 30 capsule moi</t>
         </is>
       </c>
       <c r="G9" s="132" t="n"/>
@@ -2317,7 +2317,7 @@
       </c>
       <c r="C10" s="133" t="inlineStr">
         <is>
-          <t>Flacon 200 comprimate + capac</t>
+          <t>Ambalaj interior capsule vegetale in cutie (blister sau flacon, de confirmat)</t>
         </is>
       </c>
       <c r="D10" s="133" t="inlineStr">
@@ -2327,12 +2327,12 @@
       </c>
       <c r="E10" s="133" t="inlineStr">
         <is>
-          <t>Alb (flacon si capac, din poza)</t>
+          <t>De confirmat</t>
         </is>
       </c>
       <c r="F10" s="133" t="inlineStr">
         <is>
-          <t>Spirulină 500mg 200 comprimate</t>
+          <t>5-HTP plus 30 capsule vegetale; Adaptonic 20 capsule vegetale; Adaptonic Pachet 20+20 capsule vegetale; Articlar Colagen 30 capsule vegetale; Coenzima Q10 120mg 40 capsule vegetale; Coenzima Q10 200mg Intensiv 30 capsule vegetale; Coenzima Q10 60mg 30 capsule vegetale; Coenzima Q10 Complex 30 capsule vegetale; Detenso Calm 20 capsule vegetale; Detenso Somn 30 capsule vegetale; Detoxi complet 30 capsule vegetale; Femena Meno 30 capsule vegetale; Femena Meno Pachet 30+30 capsule vegetale; Femena Osteo 30 capsule vegetale; Ginkgo biloba cu Magneziu 60 capsule vegetale; Magne 5 30 capsule vegetale; Memo Clar 60 capsule vegetale; Neuro Clar 60 capsule vegetale; Nutrinergic 30 capsule vegetale; Nutrinergic Pachet 30+30 capsule vegetale; Păr și unghii 60 capsule vegetale; Păr și Unghii Pachet 60+60 capsule vegetale; Resveratrol sincro 30 capsule vegetale; Silfide Complex de slăbit forte + Fucoidan 60 capsule vegetale; Silfide Complex de slăbit forte + Fucoidan Pachet 60+60 capsule vegetale</t>
         </is>
       </c>
       <c r="G10" s="132" t="n"/>
@@ -2362,7 +2362,7 @@
       </c>
       <c r="C11" s="133" t="inlineStr">
         <is>
-          <t>Flacon 120 capsule moi + capac</t>
+          <t>Ambalaj interior comprimate in cutie (blister sau flacon, de confirmat)</t>
         </is>
       </c>
       <c r="D11" s="133" t="inlineStr">
@@ -2372,12 +2372,12 @@
       </c>
       <c r="E11" s="133" t="inlineStr">
         <is>
-          <t>Alb (flacon si capac, din poza)</t>
+          <t>De confirmat</t>
         </is>
       </c>
       <c r="F11" s="133" t="inlineStr">
         <is>
-          <t>Ulei de somon Omega 3 120 capsule moi; Ulei de pește Omega 3 120 capsule moi; Silymarin Milk thistle 1000mg 120 capsule moi</t>
+          <t>Antistres 30 comprimate; Articlar forte 60 comprimate; Articlar Forte Pachet 60+60 comprimate; Atusin 20 comprimate; Calciu D3 masticabil 30 comprimate; Colesterol control 60 comprimate; Complex B forte 100 comprimate; Complex menopauză 30 comprimate; Control diab 60 comprimate; Curcumin 95% curcuminoide 60 comprimate; Curcumin 95% Curcuminoide Pachet 60 + 60 comprimate; Heparepar 30 comprimate; Imunio 30 comprimate; Masculin Potent 30 comprimate; Masculin Potent 30 comprimate + Ginseng siberian 30 capsule vegetale; Memorie și concentrare 30 comprimate; Montant 30 comprimate; Montant Pachet 30+30 comprimate; Optimicin 20 comprimate; Silfide Complex de slăbit forte 100 comprimate; Silfide Complex de slăbit forte 100 comprimate + Ceai de slăbit 30 plicuri; Silfide Detox 30 comprimate; Silimarină 150mg 50 comprimate; Silimarină 300mg 50 comprimate; Silimarină 300mg Pachet 50+50 comprimate; Stres Formula 30 comprimate; Vitamine și multiminerale 30 comprimate</t>
         </is>
       </c>
       <c r="G11" s="132" t="n"/>
@@ -2407,7 +2407,7 @@
       </c>
       <c r="C12" s="133" t="inlineStr">
         <is>
-          <t>Flacon 120 capsule vegetale + capac</t>
+          <t>Ambalaj interior comprimate masticabile in cutie (blister sau flacon, de confirmat)</t>
         </is>
       </c>
       <c r="D12" s="133" t="inlineStr">
@@ -2417,12 +2417,12 @@
       </c>
       <c r="E12" s="133" t="inlineStr">
         <is>
-          <t>Alb (flacon si capac, din poza)</t>
+          <t>De confirmat</t>
         </is>
       </c>
       <c r="F12" s="133" t="inlineStr">
         <is>
-          <t>Vitamina C cu Zn și D3 1000mg 120 capsule vegetale; Vitamina D3 Optim 2000UI 120 capsule vegetale; Vitamina C 1000mg 120 capsule vegetale; Articlar Colagen 120 capsule vegetale; D3 + K2 Forte 120 capsule vegetale; Magneziu 375mg B6 120 capsule vegetale; Zinc Optim 25mg 120 capsule vegetale; Magneziu Bisglicinat 120 capsule vegetale</t>
+          <t>Complex gastric 30 comprimate masticabile; Florisept 20 comprimate masticabile; Propolis C-tare 30 comprimate masticabile; Propolis Vitamina C cu Echinacea și stevie 40 comprimate masticabile</t>
         </is>
       </c>
       <c r="G12" s="132" t="n"/>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="C13" s="133" t="inlineStr">
         <is>
-          <t>Flacon 120 comprimate + capac</t>
+          <t>Flacon capsule/comprimate + capac (eticheta 215x57 mm)</t>
         </is>
       </c>
       <c r="D13" s="133" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="F13" s="133" t="inlineStr">
         <is>
-          <t>Maca Pachet 120+120 comprimate; Vitamina B12 Optim 1000µg 120 comprimate; Maca 120 comprimate</t>
+          <t>Articlar Colagen 120 capsule vegetale; D3 + K2 Forte 120 capsule vegetale; Magneziu Bisglicinat 120 capsule vegetale; Magtein® 90 capsule vegetale; Seleniu Natural 200µg 120 comprimate filmate; Silymarin Milk thistle 1000mg 120 capsule moi; Ulei de pește Omega 3 120 capsule moi; Ulei de somon Omega 3 120 capsule moi; Vitamina B12 Optim 1000µg 120 comprimate; Vitamina C 1000mg 120 capsule vegetale; Vitamina C cu Zn și D3 1000mg 120 capsule vegetale</t>
         </is>
       </c>
       <c r="G13" s="132" t="n"/>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="C14" s="133" t="inlineStr">
         <is>
-          <t>Flacon 120 comprimate filmate + capac</t>
+          <t>Flacon capsule/comprimate + capac (eticheta 180x68 mm)</t>
         </is>
       </c>
       <c r="D14" s="133" t="inlineStr">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="F14" s="133" t="inlineStr">
         <is>
-          <t>Seleniu Natural 200µg 120 comprimate filmate</t>
+          <t>Ca+D3 60 comprimate; Calciu Magneziu Zinc 100 comprimate; CaMgZn + Vitamina C 60 comprimate; Coenzima Q10 60mg 60 capsule vegetale; Coenzima Q10 cu Catină 60 comprimate; Ginkgo biloba 100mg 60 comprimate; Ginkgo biloba 100mg Pachet 60+60 comprimate; Lecitină 1200mg 60 capsule moi; Magneziu 375mg B6 120 capsule vegetale; Omega 3 6 9 60 capsule moi; Omega 3 6 9 Pachet 60+60 capsule moi; Silimarină 150mg 100 comprimate; Silimarină 300mg 100 comprimate; Silymarin Milk thistle 1000mg 60 capsule moi; Spirulină 500mg 200 comprimate; Spirulină Bio 1000mg 100 comprimate; Spirulină Bio 1000mg Pachet 100+100 comprimate; Ulei de pește Omega 3 70 capsule moi; Ulei de somon Omega 3 60 capsule moi; Vitamina D3 Optim 2000UI 120 capsule vegetale; Zinc Optim 25mg 120 capsule vegetale</t>
         </is>
       </c>
       <c r="G14" s="132" t="n"/>
@@ -2542,7 +2542,7 @@
       </c>
       <c r="C15" s="133" t="inlineStr">
         <is>
-          <t>Flacon 100 comprimate + capac</t>
+          <t>Flacon capsule/comprimate + capac (eticheta 169x58,5 mm)</t>
         </is>
       </c>
       <c r="D15" s="133" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="F15" s="133" t="inlineStr">
         <is>
-          <t>Spirulină Bio 1000mg 100 comprimate; Calciu Magneziu Zinc 100 comprimate; Zaharină 100 comprimate; Silimarină 300mg 100 comprimate; Silimarină 150mg 100 comprimate; Spirulină Bio 1000mg Pachet 100+100 comprimate</t>
+          <t>Anghinare 60 comprimate; Anghinare Pachet 60+60 comprimate; Ashwagandha KSM-66® 600mg 30 capsule vegetale; Astaxanthin 6mg 30 capsule vegetale; Berberină Duo 60 capsule vegetale; Berberină Momordica Gluco Suport 30 capsule vegetale; Ca-Mg-Zn Vitamineral 60 comprimate; Calciu citrat Vitamina D3 30 capsule vegetale; Chimen Negru 500mg 30 capsule moi; Coenzima Q10 120mg 30 capsule vegetale; Coenzima Q10 120mg Pachet 30+30 capsule vegetale; D3 + K2 30 capsule vegetale; D3 + K2 Forte 30 capsule vegetale; EnzimDigest 30 capsule vegetale; Fier lipozomal 30 capsule vegetale; L-Arginină 60 capsule vegetale; Maca 120 comprimate; Maca Pachet 120+120 comprimate; Magneziu 375mg 30 capsule vegetale; Magneziu Bisglicinat 60 capsule vegetale; Magneziu Bisglicinat Forte 30 capsule vegetale; Magneziu Bisglicinat Somn 30 capsule vegetale; Magneziu citrat 30 capsule vegetale; Melatonină 3mg 30 capsule vegetale; Melatonină 5mg 30 capsule vegetale; MSM Optim 1000mg 30 comprimate; ProstatoSan 30 capsule vegetale; Quercetin cu Zn și D3 30 capsule vegetale; Quercetin cu Zn și D3 Pachet 30+30 capsule vegetale; Rhodiola 60 comprimate; Rhodiola Pachet 60+60 comprimate; Spirulină Bio 1000mg 45 comprimate; Tămâie 500mg Boswellia serrata 60 capsule vegetale; Vitamina C 1000mg 30 capsule vegetale; Vitamina C cu Zn și D3 1000mg 30 capsule vegetale; Vitamina C Lipozomală 30 capsule vegetale; Zinc bisglicinat 30 capsule vegetale</t>
         </is>
       </c>
       <c r="G15" s="132" t="n"/>
@@ -2587,7 +2587,7 @@
       </c>
       <c r="C16" s="133" t="inlineStr">
         <is>
-          <t>Flacon 90 capsule vegetale + capac</t>
+          <t>Flacon capsule/comprimate + capac (eticheta 140x46 mm)</t>
         </is>
       </c>
       <c r="D16" s="133" t="inlineStr">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="F16" s="133" t="inlineStr">
         <is>
-          <t>Magtein® 90 capsule vegetale</t>
+          <t>Calciu lactic 30 comprimate; Calciu lactic 60 comprimate; Calciu Magneziu D 30 comprimate; Calciu Magneziu D Pachet 30+30 comprimate; Calciu Magneziu Zinc 40 comprimate; Calciu Vitamina D3 40 comprimate; Complex B 30 comprimate; Magneziu Vitamina B6 30 comprimate; Seleniu Natural 200µg 30 comprimate filmate; Urifin 30 comprimate; Urifin 30 comprimate + Urifin Ceai 20 plicuri; Urifin Pachet 30+30 comprimate; Vitamina B12 Optim 1000µg 30 comprimate; Vitamina C 180mg 20 comprimate masticabile; Vitamina C 180mg 60 comprimate masticabile; Vitamina D3 Forte 5000UI 30 comprimate; Vitamina D3 Optim 2000UI 30 capsule vegetale; Vitamine și minerale esențiale 30 comprimate; Zaharină 100 comprimate; Zinc Optim 25mg 30 capsule vegetale</t>
         </is>
       </c>
       <c r="G16" s="132" t="n"/>
@@ -2632,7 +2632,7 @@
       </c>
       <c r="C17" s="133" t="inlineStr">
         <is>
-          <t>Flacon 70 capsule moi + capac</t>
+          <t>Flacon capsule/comprimate + capac (eticheta 99x14 mm)</t>
         </is>
       </c>
       <c r="D17" s="133" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="F17" s="133" t="inlineStr">
         <is>
-          <t>Ulei de pește Omega 3 70 capsule moi</t>
+          <t>Bomboane cu mentă 60 comprimate masticabile</t>
         </is>
       </c>
       <c r="G17" s="132" t="n"/>
@@ -2677,7 +2677,7 @@
       </c>
       <c r="C18" s="133" t="inlineStr">
         <is>
-          <t>Flacon 60 capsule moi + capac</t>
+          <t>Flacon brun capsule/comprimate + capac (eticheta 169x58,5 mm)</t>
         </is>
       </c>
       <c r="D18" s="133" t="inlineStr">
@@ -2687,12 +2687,12 @@
       </c>
       <c r="E18" s="133" t="inlineStr">
         <is>
-          <t>Alb (flacon si capac, din poza)</t>
+          <t>Brun (flacon), maro (capac), din poza</t>
         </is>
       </c>
       <c r="F18" s="133" t="inlineStr">
         <is>
-          <t>Ulei de somon Omega 3 60 capsule moi; Lecitină 1200mg 60 capsule moi; Omega 3 6 9 Pachet 60+60 capsule moi; Omega 3 6 9 60 capsule moi; Silymarin Milk thistle 1000mg 60 capsule moi</t>
+          <t>Ginkana Circulație 30 capsule vegetale; Ginkana Memorie 30 capsule vegetale; Ginkana Memorie 30+30 capsule vegetale</t>
         </is>
       </c>
       <c r="G18" s="132" t="n"/>
@@ -2722,7 +2722,7 @@
       </c>
       <c r="C19" s="133" t="inlineStr">
         <is>
-          <t>Flacon 60 capsule vegetale + capac</t>
+          <t>Flacon brun capsule/comprimate + capac (eticheta 140x46 mm)</t>
         </is>
       </c>
       <c r="D19" s="133" t="inlineStr">
@@ -2732,12 +2732,12 @@
       </c>
       <c r="E19" s="133" t="inlineStr">
         <is>
-          <t>Alb (flacon si capac, din poza)</t>
+          <t>Brun (flacon), maro (capac), din poza</t>
         </is>
       </c>
       <c r="F19" s="133" t="inlineStr">
         <is>
-          <t>Tămâie 500mg Boswellia serrata 60 capsule vegetale; L-Arginină 60 capsule vegetale; Berberină Duo 60 capsule vegetale; Coenzima Q10 60mg 60 capsule vegetale; Magneziu Bisglicinat 60 capsule vegetale</t>
+          <t>Ginkana Ginkgo biloba 120mg 30 comprimate; Ginkana Ginkgo biloba 120mg Pachet 30+30 comprimate; Ginkana Ginkgo biloba 40mg 30 comprimate; Ginkana Ginkgo biloba 40mg Pachet 30+30 comprimate; Ginkana Ginkgo biloba 80mg forte 30 comprimate; Ginkana Ginkgo biloba 80mg forte Pachet 30+30 comprimate; Ginseng 30 comprimate; Ginseng Pachet 30+30 comprimate; Ginseng siberian 30 capsule vegetale; Ginseng siberian Pachet 30+30 capsule vegetale; Masculin Potent 30 comprimate + Ginseng siberian 30 capsule vegetale; Spirulină 500mg 30 comprimate; Spirulină 500mg Pachet 30+30 comprimate</t>
         </is>
       </c>
       <c r="G19" s="132" t="n"/>
@@ -2767,22 +2767,22 @@
       </c>
       <c r="C20" s="133" t="inlineStr">
         <is>
-          <t>Flacon 60 comprimate + capac</t>
+          <t>Flacon 1000 ml + capac</t>
         </is>
       </c>
       <c r="D20" s="133" t="inlineStr">
         <is>
-          <t>De confirmat</t>
+          <t>1000 ml</t>
         </is>
       </c>
       <c r="E20" s="133" t="inlineStr">
         <is>
-          <t>Alb (flacon si capac, din poza)</t>
+          <t>Alb (din poza)</t>
         </is>
       </c>
       <c r="F20" s="133" t="inlineStr">
         <is>
-          <t>Ginkgo biloba 100mg Pachet 60+60 comprimate; Rhodiola Pachet 60+60 comprimate; Anghinare 60 comprimate; Calciu lactic 60 comprimate; Anghinare Pachet 60+60 comprimate; Ca-Mg-Zn Vitamineral 60 comprimate; Ca+D3 60 comprimate; CaMgZn + Vitamina C 60 comprimate; Ginkgo biloba 100mg 60 comprimate; Coenzima Q10 cu Catină 60 comprimate; Rhodiola 60 comprimate</t>
+          <t>Suc de Noni Tahitian Bio 1000ml; Suc ecologic de Aloe Vera 1000ml</t>
         </is>
       </c>
       <c r="G20" s="132" t="n"/>
@@ -2812,22 +2812,22 @@
       </c>
       <c r="C21" s="133" t="inlineStr">
         <is>
-          <t>Flacon 60 comprimate masticabile + capac</t>
+          <t>Flacon 150 ml + capac (plastic sau sticla, de confirmat)</t>
         </is>
       </c>
       <c r="D21" s="133" t="inlineStr">
         <is>
+          <t>150 ml</t>
+        </is>
+      </c>
+      <c r="E21" s="133" t="inlineStr">
+        <is>
           <t>De confirmat</t>
         </is>
       </c>
-      <c r="E21" s="133" t="inlineStr">
-        <is>
-          <t>Alb (flacon si capac, din poza)</t>
-        </is>
-      </c>
       <c r="F21" s="133" t="inlineStr">
         <is>
-          <t>Bomboane cu mentă 60 comprimate masticabile; Vitamina C 180mg 60 comprimate masticabile</t>
+          <t>Atusin Sirop 150ml; Dodino Sirop Atusin 150ml; Dodino Sirop Calciu și Vitamina D3 150ml; Dodino Sirop cu Magneziu și Complex B 150ml; Dodino Sirop de Propolis cu Echinacea 150ml; Dodino Sirop Memorie și Concentrare 150ml; Dodino Sirop Vermilin 150ml; Dodino Sirop Vitamine și Multiminerale 150ml; Gripalin Sirop 150ml; Sirop de muguri de pin și brad 150ml; Sirop de pătlagină 150ml; Sirop laxatin 150ml; Sirop pentru imunitate 150ml; Sirop pentru somn 150ml</t>
         </is>
       </c>
       <c r="G21" s="132" t="n"/>
@@ -2857,22 +2857,22 @@
       </c>
       <c r="C22" s="133" t="inlineStr">
         <is>
-          <t>Flacon 45 comprimate + capac</t>
+          <t>Flacon 20 ml + spray (plastic sau sticla, de confirmat)</t>
         </is>
       </c>
       <c r="D22" s="133" t="inlineStr">
         <is>
+          <t>20 ml</t>
+        </is>
+      </c>
+      <c r="E22" s="133" t="inlineStr">
+        <is>
           <t>De confirmat</t>
         </is>
       </c>
-      <c r="E22" s="133" t="inlineStr">
-        <is>
-          <t>Alb (flacon si capac, din poza)</t>
-        </is>
-      </c>
       <c r="F22" s="133" t="inlineStr">
         <is>
-          <t>Spirulină Bio 1000mg 45 comprimate</t>
+          <t>Propolis C-tare Spray 20ml</t>
         </is>
       </c>
       <c r="G22" s="132" t="n"/>
@@ -2902,7 +2902,7 @@
       </c>
       <c r="C23" s="133" t="inlineStr">
         <is>
-          <t>Flacon 40 comprimate + capac</t>
+          <t>Plic monodoza pulbere solubila</t>
         </is>
       </c>
       <c r="D23" s="133" t="inlineStr">
@@ -2912,12 +2912,12 @@
       </c>
       <c r="E23" s="133" t="inlineStr">
         <is>
-          <t>Alb (flacon si capac, din poza)</t>
+          <t>De confirmat</t>
         </is>
       </c>
       <c r="F23" s="133" t="inlineStr">
         <is>
-          <t>Calciu Magneziu Zinc 40 comprimate; Calciu Vitamina D3 40 comprimate</t>
+          <t>Articlar HyaluCollagen Solubil 20 plicuri; Articlar HyaluCollagen Solubil 30 plicuri; Beauty HyaluCollagen Solubil 20 plicuri; Calciu 1200mg Vitamina D3 Solubil 20 plicuri; Calciu Magneziu Zinc D3 Solubil 20 plicuri; Electroliți Forte - Săruri de rehidratare Solubil 20 plicuri; Gripalin Natural Solubil 10 plicuri; Magneziu 300mg Solubil 20 plicuri; Urifin rapid Solubil 15 plicuri; Urifin Rapid Solubil 15 plicuri + Ceai Urifin 20 plicuri Pachet x 2; Vitamina C Naturală 1000mg Solubil 15 plicuri; Vitamine și minerale Forte Solubil 15 plicuri</t>
         </is>
       </c>
       <c r="G23" s="132" t="n"/>
@@ -2947,22 +2947,22 @@
       </c>
       <c r="C24" s="133" t="inlineStr">
         <is>
-          <t>Flacon 30 capsule moi + capac</t>
+          <t>Borcan 250 g + capac</t>
         </is>
       </c>
       <c r="D24" s="133" t="inlineStr">
         <is>
-          <t>De confirmat</t>
+          <t>250 g / 250 ml</t>
         </is>
       </c>
       <c r="E24" s="133" t="inlineStr">
         <is>
-          <t>Alb (flacon si capac, din poza)</t>
+          <t>Alb (borcan si capac, din poza)</t>
         </is>
       </c>
       <c r="F24" s="133" t="inlineStr">
         <is>
-          <t>Chimen Negru 500mg 30 capsule moi</t>
+          <t>Articlar Gel 250g; Balsam Puterea Calului cu chili 250g; Balsam Vigoarea Ursului Polar 250g; Cremă de Arnică 250 ml; Cremă de Gălbenele 250g; Gheara Diavolului Balsam 250g; Gheara Diavolului Canabis Gel 250g; Picioare Obosite Cremă 250g; Puterea Calului Canabis Gel 250g</t>
         </is>
       </c>
       <c r="G24" s="132" t="n"/>
@@ -2992,22 +2992,22 @@
       </c>
       <c r="C25" s="133" t="inlineStr">
         <is>
-          <t>Flacon 30 capsule vegetale + capac</t>
+          <t>Recipient pulbere 300 g + capac</t>
         </is>
       </c>
       <c r="D25" s="133" t="inlineStr">
         <is>
-          <t>De confirmat</t>
+          <t>300 g</t>
         </is>
       </c>
       <c r="E25" s="133" t="inlineStr">
         <is>
-          <t>Alb (flacon si capac, din poza)</t>
+          <t>Alb (din poza)</t>
         </is>
       </c>
       <c r="F25" s="133" t="inlineStr">
         <is>
-          <t>Vitamina D3 Optim 2000UI 30 capsule vegetale; D3 + K2 30 capsule vegetale; Vitamina C 1000mg 30 capsule vegetale; Fier lipozomal 30 capsule vegetale; Berberină Momordica Gluco Suport 30 capsule vegetale; Coenzima Q10 120mg Pachet 30+30 capsule vegetale; Zinc bisglicinat 30 capsule vegetale; ProstatoSan 30 capsule vegetale; Magneziu Bisglicinat Forte 30 capsule vegetale; D3 + K2 Forte 30 capsule vegetale; EnzimDigest 30 capsule vegetale; Melatonină 3mg 30 capsule vegetale; Calciu citrat Vitamina D3 30 capsule vegetale; Melatonină 5mg 30 capsule vegetale; Vitamina C cu Zn și D3 1000mg 30 capsule vegetale; Quercetin cu Zn și D3 Pachet 30+30 capsule vegetale; Vitamina C Lipozomală 30 capsule vegetale; Magneziu citrat 30 capsule vegetale; Zinc Optim 25mg 30 capsule vegetale; Magneziu 375mg 30 capsule vegetale; Quercetin cu Zn și D3 30 capsule vegetale; Coenzima Q10 120mg 30 capsule vegetale; Astaxanthin 6mg 30 capsule vegetale; Ashwagandha KSM-66® 600mg 30 capsule vegetale; Magneziu Bisglicinat Somn 30 capsule vegetale</t>
+          <t>Colagen Peptide 300g; Colagen Peptide cu Acid hialuronic și Vitamina C 300g</t>
         </is>
       </c>
       <c r="G25" s="132" t="n"/>
@@ -3037,22 +3037,22 @@
       </c>
       <c r="C26" s="133" t="inlineStr">
         <is>
-          <t>Flacon 30 comprimate + capac</t>
+          <t>Recipient pulbere 140 g + capac</t>
         </is>
       </c>
       <c r="D26" s="133" t="inlineStr">
         <is>
-          <t>De confirmat</t>
+          <t>140 g</t>
         </is>
       </c>
       <c r="E26" s="133" t="inlineStr">
         <is>
-          <t>Alb (flacon si capac, din poza)</t>
+          <t>Alb (din poza)</t>
         </is>
       </c>
       <c r="F26" s="133" t="inlineStr">
         <is>
-          <t>Magneziu Vitamina B6 30 comprimate; Vitamina D3 Forte 5000UI 30 comprimate; MSM Optim 1000mg 30 comprimate; Urifin Pachet 30+30 comprimate; Vitamina B12 Optim 1000µg 30 comprimate; Calciu Magneziu D Pachet 30+30 comprimate; Calciu lactic 30 comprimate; Calciu Magneziu D 30 comprimate; Complex B 30 comprimate; Vitamine și minerale esențiale 30 comprimate; Urifin 30 comprimate</t>
+          <t>Inulină 140g</t>
         </is>
       </c>
       <c r="G26" s="132" t="n"/>
@@ -3082,22 +3082,22 @@
       </c>
       <c r="C27" s="133" t="inlineStr">
         <is>
-          <t>Flacon 30 comprimate filmate + capac</t>
+          <t>Borcan 20 g + capac</t>
         </is>
       </c>
       <c r="D27" s="133" t="inlineStr">
         <is>
-          <t>De confirmat</t>
+          <t>20 g</t>
         </is>
       </c>
       <c r="E27" s="133" t="inlineStr">
         <is>
-          <t>Alb (flacon si capac, din poza)</t>
+          <t>Alb (din poza)</t>
         </is>
       </c>
       <c r="F27" s="133" t="inlineStr">
         <is>
-          <t>Seleniu Natural 200µg 30 comprimate filmate</t>
+          <t>Alifie chinezească 20g; Balsam Arnică 20g; Balsam călcâie 20g; Balsam Gălbenele 20g; Balsam Gălbenele și Tătăneasă 20g; Balsam Propolis 20g; Balsam Rostopască 20g; Balsam Tătăneasă 20g</t>
         </is>
       </c>
       <c r="G27" s="132" t="n"/>
@@ -3127,22 +3127,22 @@
       </c>
       <c r="C28" s="133" t="inlineStr">
         <is>
-          <t>Flacon 20 comprimate masticabile + capac</t>
+          <t>Tub 200 ml + capac</t>
         </is>
       </c>
       <c r="D28" s="133" t="inlineStr">
         <is>
-          <t>De confirmat</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="E28" s="133" t="inlineStr">
         <is>
-          <t>Alb (flacon si capac, din poza)</t>
+          <t>Alb (din poza)</t>
         </is>
       </c>
       <c r="F28" s="133" t="inlineStr">
         <is>
-          <t>Vitamina C 180mg 20 comprimate masticabile</t>
+          <t>Gel anticelulitic 200ml</t>
         </is>
       </c>
       <c r="G28" s="132" t="n"/>
@@ -3172,22 +3172,22 @@
       </c>
       <c r="C29" s="133" t="inlineStr">
         <is>
-          <t>Flacon 30 capsule vegetale + capac</t>
+          <t>Tub 150 ml + capac</t>
         </is>
       </c>
       <c r="D29" s="133" t="inlineStr">
         <is>
-          <t>De confirmat</t>
+          <t>150 ml</t>
         </is>
       </c>
       <c r="E29" s="133" t="inlineStr">
         <is>
-          <t>Brun (flacon), maro (capac), din poza</t>
+          <t>Alb (din poza)</t>
         </is>
       </c>
       <c r="F29" s="133" t="inlineStr">
         <is>
-          <t>Ginkana Memorie 30 capsule vegetale; Ginseng siberian Pachet 30+30 capsule vegetale; Ginkana Circulație 30 capsule vegetale; Ginseng siberian 30 capsule vegetale; Ginkana Memorie 30+30 capsule vegetale; Masculin Potent 30 comprimate + Ginseng siberian 30 capsule vegetale</t>
+          <t>Cremă antivergeturi 150ml</t>
         </is>
       </c>
       <c r="G29" s="132" t="n"/>
@@ -3217,22 +3217,22 @@
       </c>
       <c r="C30" s="133" t="inlineStr">
         <is>
-          <t>Flacon 30 comprimate + capac</t>
+          <t>Tub 50 ml + capac</t>
         </is>
       </c>
       <c r="D30" s="133" t="inlineStr">
         <is>
-          <t>De confirmat</t>
+          <t>50 ml</t>
         </is>
       </c>
       <c r="E30" s="133" t="inlineStr">
         <is>
-          <t>Brun (flacon), maro (capac), din poza</t>
+          <t>Alb (din poza)</t>
         </is>
       </c>
       <c r="F30" s="133" t="inlineStr">
         <is>
-          <t>Ginkana Ginkgo biloba 80mg forte Pachet 30+30 comprimate; Ginseng Pachet 30+30 comprimate; Ginkana Ginkgo biloba 40mg Pachet 30+30 comprimate; Spirulină 500mg Pachet 30+30 comprimate; Ginkana Ginkgo biloba 120mg Pachet 30+30 comprimate; Ginkana Ginkgo biloba 80mg forte 30 comprimate; Ginkana Ginkgo biloba 40mg 30 comprimate; Ginkana Ginkgo biloba 120mg 30 comprimate; Ginseng 30 comprimate; Spirulină 500mg 30 comprimate</t>
+          <t>Articlar Gel 50ml; Crema cu uree 15% 50ml; Cremă de mâini cu Gălbenele și Aloe vera 50ml; Gel înțepături insecte 50ml</t>
         </is>
       </c>
       <c r="G30" s="132" t="n"/>
@@ -3262,12 +3262,12 @@
       </c>
       <c r="C31" s="133" t="inlineStr">
         <is>
-          <t>Flacon 1000 ml + capac</t>
+          <t>Tub 20 ml + capac</t>
         </is>
       </c>
       <c r="D31" s="133" t="inlineStr">
         <is>
-          <t>1000 ml</t>
+          <t>20 ml</t>
         </is>
       </c>
       <c r="E31" s="133" t="inlineStr">
@@ -3277,7 +3277,7 @@
       </c>
       <c r="F31" s="133" t="inlineStr">
         <is>
-          <t>Suc de Noni Tahitian Bio 1000ml; Suc ecologic de Aloe Vera 1000ml</t>
+          <t>Cremă Antiacneică 20 ml; Gel bătături 20ml</t>
         </is>
       </c>
       <c r="G31" s="132" t="n"/>
@@ -3307,12 +3307,12 @@
       </c>
       <c r="C32" s="133" t="inlineStr">
         <is>
-          <t>Flacon 20 ml + spray (in cutie)</t>
+          <t>Plic ceai (in cutie)</t>
         </is>
       </c>
       <c r="D32" s="133" t="inlineStr">
         <is>
-          <t>20 ml</t>
+          <t>De confirmat</t>
         </is>
       </c>
       <c r="E32" s="133" t="inlineStr">
@@ -3322,7 +3322,7 @@
       </c>
       <c r="F32" s="133" t="inlineStr">
         <is>
-          <t>Propolis C-tare Spray 20ml</t>
+          <t>Atusin Ceai 20 plicuri; Ceai antigripol 40 plicuri; Ceai antistres 20 plicuri; Ceai colesterol 20 plicuri; Ceai cu afine 20 plicuri; Ceai cu mere și coacăze 20 plicuri; Ceai de crușin 20 plicuri; Ceai de ghimbir cu coajă de portocale 20 plicuri; Ceai de gălbenele 20 plicuri; Ceai de gălbenele 40 plicuri; Ceai de lavandă 20 plicuri; Ceai de mentă 20 plicuri; Ceai de mentă cu aromă de lămâie 20 plicuri; Ceai de mușețel 20 plicuri; Ceai de mușețel 40 plicuri; Ceai de slăbit 20 plicuri; Ceai de slăbit 40 plicuri; Ceai de soc 20 plicuri; Ceai de sunătoare 20 plicuri; Ceai de sunătoare 40 plicuri; Ceai de tei 20 plicuri; Ceai de tei 40 plicuri; Ceai de urzică 20 plicuri; Ceai digestiv 20 plicuri; Ceai diuretic 20 plicuri; Ceai fructe de pădure 20 plicuri; Ceai gastric 20 plicuri; Ceai Gripalin 20 plicuri; Ceai hepatic 20 plicuri; Ceai hepatic 40 plicuri; Ceai imunitate 20 plicuri; Ceai laxatin 20 plicuri; Ceai menopauză 20 plicuri; Ceai negru 20 plicuri; Ceai normalizarea glicemiei 20 plicuri; Ceai normalizarea glicemiei 40 plicuri; Ceai pentru articulații 20 plicuri; Ceai pentru prostată 20 plicuri; Ceai pentru somn 20 plicuri; Ceai pentru tensiune 20 plicuri; Ceai renal 20 plicuri; Ceai verde 20 plicuri; Complex de slăbit ceai cu ginseng și ananas 30 plicuri; Silfide Complex de slăbit forte 100 comprimate + Ceai de slăbit 30 plicuri; Urifin 30 comprimate + Urifin Ceai 20 plicuri; Urifin Rapid Solubil 15 plicuri + Ceai Urifin 20 plicuri Pachet x 2</t>
         </is>
       </c>
       <c r="G32" s="132" t="n"/>
@@ -3352,22 +3352,22 @@
       </c>
       <c r="C33" s="133" t="inlineStr">
         <is>
-          <t>Recipient pulbere 300 g + capac</t>
+          <t>Plic piramida ceai (in cutie)</t>
         </is>
       </c>
       <c r="D33" s="133" t="inlineStr">
         <is>
-          <t>300 g</t>
+          <t>De confirmat</t>
         </is>
       </c>
       <c r="E33" s="133" t="inlineStr">
         <is>
-          <t>Alb (din poza)</t>
+          <t>De confirmat</t>
         </is>
       </c>
       <c r="F33" s="133" t="inlineStr">
         <is>
-          <t>Colagen Peptide 300g; Colagen Peptide cu Acid hialuronic și Vitamina C 300g</t>
+          <t>TABIETURI Ceai de Fructe roșii 12 plicuri; TABIETURI Ceai de Mentă delicat 12 plicuri; TABIETURI Ceai de Merișor 12 plicuri; TABIETURI Ceai de Mușețel și citrice 12 plicuri; TABIETURI Ceai English breakfast 12 plicuri; TABIETURI Ceai Fruit melange 12 plicuri; TABIETURI Ceai Oriental condimentat 12 plicuri; TABIETURI Ceai Rooibos Creme brulee 12 plicuri; TABIETURI Ceai Verde cu aromă de Iasomie 12 plicuri</t>
         </is>
       </c>
       <c r="G33" s="132" t="n"/>
@@ -3397,22 +3397,22 @@
       </c>
       <c r="C34" s="133" t="inlineStr">
         <is>
-          <t>Borcan 250 g + capac</t>
+          <t>Punga interioara ceai vrac (in cutie, de confirmat)</t>
         </is>
       </c>
       <c r="D34" s="133" t="inlineStr">
         <is>
-          <t>250 g / 250 ml</t>
+          <t>40 / 50 / 70 g</t>
         </is>
       </c>
       <c r="E34" s="133" t="inlineStr">
         <is>
-          <t>Alb (borcan si capac, din poza)</t>
+          <t>De confirmat</t>
         </is>
       </c>
       <c r="F34" s="133" t="inlineStr">
         <is>
-          <t>Picioare Obosite Cremă 250g; Balsam Vigoarea Ursului Polar 250g; Gheara Diavolului Balsam 250g; Cremă de Gălbenele 250g; Cremă de Arnică 250 ml; Balsam Puterea Calului cu chili 250g; Articlar Gel 250g; Puterea Calului Canabis Gel 250g; Gheara Diavolului Canabis Gel 250g</t>
+          <t>Ceai de anason vrac 50g; Ceai de anghinare vrac 50g; Ceai de armurariu vrac 50g; Ceai de chimen vrac 50g; Ceai de coada calului vrac 50g; Ceai de coada șoricelului vrac 50g; Ceai de codițe de cireșe vrac 50g; Ceai de cătină vrac 50g; Ceai de echinacea vrac 50g; Ceai de fenicul vrac 50g; Ceai de ghimbir vrac 50g; Ceai de ghimpe vrac 50g; Ceai de gălbenele vrac 50g; Ceai de lemn-dulce vrac 40g; Ceai de mentă vrac 50g; Ceai de mușețel vrac 40g; Ceai de măceșe vrac 50g; Ceai de pufuliță cu flori mici vrac 50g; Ceai de păducel cu flori vrac 50g; Ceai de păpădie vrac 50g; Ceai de pătlagină vrac 50g; Ceai de roinița vrac 50g; Ceai de salvie vrac 50g; Ceai de senna vrac 50g; Ceai de slăbit vrac 50g; Ceai de sunătoare vrac 50g; Ceai de tei vrac 40g; Ceai detoxifiere vrac 50g; Ceai din mătase de porumb vrac 50g; Ceai hepatobiliar vrac 50g; Ceai normalizarea glicemiei vrac 50g; Ceai pentru fiere și rinichi vrac 50 g; Complex de slăbit cu ceai verde și lămâie vrac 70g; Gripalin Ceai vrac 50g</t>
         </is>
       </c>
       <c r="G34" s="132" t="n"/>
@@ -3442,22 +3442,22 @@
       </c>
       <c r="C35" s="133" t="inlineStr">
         <is>
-          <t>Recipient pulbere 140 g + capac</t>
+          <t>Punga ceai 35 g</t>
         </is>
       </c>
       <c r="D35" s="133" t="inlineStr">
         <is>
-          <t>140 g</t>
+          <t>35 g</t>
         </is>
       </c>
       <c r="E35" s="133" t="inlineStr">
         <is>
-          <t>Alb (din poza)</t>
+          <t>De confirmat</t>
         </is>
       </c>
       <c r="F35" s="133" t="inlineStr">
         <is>
-          <t>Inulină 140g</t>
+          <t>Ceai Fructe de pădure cu scorțișoară 35g; Ceai Rooibos cu vanilie 35g</t>
         </is>
       </c>
       <c r="G35" s="132" t="n"/>
@@ -3487,22 +3487,22 @@
       </c>
       <c r="C36" s="133" t="inlineStr">
         <is>
-          <t>Borcan 20 g + capac</t>
+          <t>Punga 1 kg</t>
         </is>
       </c>
       <c r="D36" s="133" t="inlineStr">
         <is>
-          <t>20 g</t>
+          <t>1 kg</t>
         </is>
       </c>
       <c r="E36" s="133" t="inlineStr">
         <is>
-          <t>Alb (din poza)</t>
+          <t>Transparenta + eticheta (din poza)</t>
         </is>
       </c>
       <c r="F36" s="133" t="inlineStr">
         <is>
-          <t>Balsam Gălbenele și Tătăneasă 20g; Alifie chinezească 20g; Balsam Propolis 20g; Balsam călcâie 20g; Balsam Rostopască 20g; Balsam Gălbenele 20g; Balsam Arnică 20g; Balsam Tătăneasă 20g</t>
+          <t>Goji 1kg; Merișor 1kg; Omega Mix 1kg; Seminte de In 1kg; Semințe de Chia 1kg; Vitamin Mix Merișor și Goji 1kg</t>
         </is>
       </c>
       <c r="G36" s="132" t="n"/>
@@ -3532,22 +3532,22 @@
       </c>
       <c r="C37" s="133" t="inlineStr">
         <is>
-          <t>Tub 200 ml + capac</t>
+          <t>Punga 500 g</t>
         </is>
       </c>
       <c r="D37" s="133" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>500 g</t>
         </is>
       </c>
       <c r="E37" s="133" t="inlineStr">
         <is>
-          <t>Alb (din poza)</t>
+          <t>Transparenta + eticheta (din poza)</t>
         </is>
       </c>
       <c r="F37" s="133" t="inlineStr">
         <is>
-          <t>Gel anticelulitic 200ml</t>
+          <t>Fulgi de Grâu 500g; Fulgi de Orz 500g; Fulgi de Ovăz 500g; Fulgi de Porumb 500g; Fulgi de Porumb fără zahăr 500g; Fulgi de Secară 500g; Goji 500g; Merișor 500g; Musli cereale și fructe uscate 500g; Musli mix 500g; Năut 500g; Omega Mix 500g; Sare roz de Himalaya Cristale neiodată 500g; Seminte de Chia 500g; Seminte de In 500g; Vitamin Mix Merisor și Goji 500g</t>
         </is>
       </c>
       <c r="G37" s="132" t="n"/>
@@ -3577,22 +3577,22 @@
       </c>
       <c r="C38" s="133" t="inlineStr">
         <is>
-          <t>Tub 150 ml + capac</t>
+          <t>Punga 250 g</t>
         </is>
       </c>
       <c r="D38" s="133" t="inlineStr">
         <is>
-          <t>150 ml</t>
+          <t>250 g</t>
         </is>
       </c>
       <c r="E38" s="133" t="inlineStr">
         <is>
-          <t>Alb (din poza)</t>
+          <t>Transparenta + eticheta (din poza)</t>
         </is>
       </c>
       <c r="F38" s="133" t="inlineStr">
         <is>
-          <t>Cremă antivergeturi 150ml</t>
+          <t>Caju crud 250g; Goji 250g; Merișor 250g; Migdale crude 250 g; Seminte Crude de Floarea Soarelui 250g; Semințe crude de Dovleac 250g; Tărâțe de Psyllium 250g</t>
         </is>
       </c>
       <c r="G38" s="132" t="n"/>
@@ -3622,22 +3622,22 @@
       </c>
       <c r="C39" s="133" t="inlineStr">
         <is>
-          <t>Tub 50 ml + capac</t>
+          <t>Punga 160 g</t>
         </is>
       </c>
       <c r="D39" s="133" t="inlineStr">
         <is>
-          <t>50 ml</t>
+          <t>160 g</t>
         </is>
       </c>
       <c r="E39" s="133" t="inlineStr">
         <is>
-          <t>Alb (din poza)</t>
+          <t>Transparenta + eticheta (din poza)</t>
         </is>
       </c>
       <c r="F39" s="133" t="inlineStr">
         <is>
-          <t>Gel înțepături insecte 50ml; Articlar Gel 50ml; Cremă de mâini cu Gălbenele și Aloe vera 50ml; Crema cu uree 15% 50ml</t>
+          <t>Seminte Crude de Floarea Soarelui 160g</t>
         </is>
       </c>
       <c r="G39" s="132" t="n"/>
@@ -3667,22 +3667,22 @@
       </c>
       <c r="C40" s="133" t="inlineStr">
         <is>
-          <t>Tub 20 ml + capac</t>
+          <t>Punga 150 g</t>
         </is>
       </c>
       <c r="D40" s="133" t="inlineStr">
         <is>
-          <t>20 ml</t>
+          <t>150 g</t>
         </is>
       </c>
       <c r="E40" s="133" t="inlineStr">
         <is>
-          <t>Alb (din poza)</t>
+          <t>Transparenta + eticheta (din poza)</t>
         </is>
       </c>
       <c r="F40" s="133" t="inlineStr">
         <is>
-          <t>Gel bătături 20ml; Cremă Antiacneică 20 ml</t>
+          <t>Arahide crude 150g; Mix Semințe de Floarea Soarelui și Dovleac 150g; Semințe crude de Dovleac 150g</t>
         </is>
       </c>
       <c r="G40" s="132" t="n"/>
@@ -3712,12 +3712,12 @@
       </c>
       <c r="C41" s="133" t="inlineStr">
         <is>
-          <t>Punga 1 kg</t>
+          <t>Punga 140 g</t>
         </is>
       </c>
       <c r="D41" s="133" t="inlineStr">
         <is>
-          <t>1 kg</t>
+          <t>140 g</t>
         </is>
       </c>
       <c r="E41" s="133" t="inlineStr">
@@ -3727,7 +3727,7 @@
       </c>
       <c r="F41" s="133" t="inlineStr">
         <is>
-          <t>Seminte de In 1kg; Merișor 1kg; Semințe de Chia 1kg; Omega Mix 1kg; Vitamin Mix Merișor și Goji 1kg; Goji 1kg</t>
+          <t>Migdale crude 140 g</t>
         </is>
       </c>
       <c r="G41" s="132" t="n"/>
@@ -3757,12 +3757,12 @@
       </c>
       <c r="C42" s="133" t="inlineStr">
         <is>
-          <t>Punga 500 g</t>
+          <t>Punga 130 g</t>
         </is>
       </c>
       <c r="D42" s="133" t="inlineStr">
         <is>
-          <t>500 g</t>
+          <t>130 g</t>
         </is>
       </c>
       <c r="E42" s="133" t="inlineStr">
@@ -3772,7 +3772,7 @@
       </c>
       <c r="F42" s="133" t="inlineStr">
         <is>
-          <t>Seminte de Chia 500g; Fulgi de Ovăz 500g; Musli cereale și fructe uscate 500g; Sare roz de Himalaya Cristale neiodată 500g; Musli mix 500g; Seminte de In 500g; Fulgi de Porumb 500g; Fulgi de Porumb fără zahăr 500g; Omega Mix 500g; Fulgi de Secară 500g; Fulgi de Grâu 500g; Vitamin Mix Merisor și Goji 500g; Goji 500g; Năut 500g; Merișor 500g; Fulgi de Orz 500g</t>
+          <t>Fistic crud 130g; Mix Caju și Migdale 130g; Mix Fructe uscate și Nuci 130g; Omega Mix 130g; Semințe de In 130g; Stafide brune 130g</t>
         </is>
       </c>
       <c r="G42" s="132" t="n"/>
@@ -3802,12 +3802,12 @@
       </c>
       <c r="C43" s="133" t="inlineStr">
         <is>
-          <t>Punga 250 g</t>
+          <t>Punga 110 g</t>
         </is>
       </c>
       <c r="D43" s="133" t="inlineStr">
         <is>
-          <t>250 g</t>
+          <t>110 g</t>
         </is>
       </c>
       <c r="E43" s="133" t="inlineStr">
@@ -3817,7 +3817,7 @@
       </c>
       <c r="F43" s="133" t="inlineStr">
         <is>
-          <t>Seminte Crude de Floarea Soarelui 250g; Migdale crude 250 g; Tărâțe de Psyllium 250g; Caju crud 250g; Merișor 250g; Semințe crude de Dovleac 250g; Goji 250g</t>
+          <t>Caju crud 110g; Merișor 110g; Vitamin Mix Merișor și Goji 110g</t>
         </is>
       </c>
       <c r="G43" s="132" t="n"/>
@@ -3847,12 +3847,12 @@
       </c>
       <c r="C44" s="133" t="inlineStr">
         <is>
-          <t>Punga 160 g</t>
+          <t>Punga 100 g</t>
         </is>
       </c>
       <c r="D44" s="133" t="inlineStr">
         <is>
-          <t>160 g</t>
+          <t>100 g</t>
         </is>
       </c>
       <c r="E44" s="133" t="inlineStr">
@@ -3862,7 +3862,7 @@
       </c>
       <c r="F44" s="133" t="inlineStr">
         <is>
-          <t>Seminte Crude de Floarea Soarelui 160g</t>
+          <t>Goji 100g; Semințe de Chia 100g; Semințe de Susan 100g</t>
         </is>
       </c>
       <c r="G44" s="132" t="n"/>
@@ -3892,12 +3892,12 @@
       </c>
       <c r="C45" s="133" t="inlineStr">
         <is>
-          <t>Punga 150 g</t>
+          <t>Punga 85 g</t>
         </is>
       </c>
       <c r="D45" s="133" t="inlineStr">
         <is>
-          <t>150 g</t>
+          <t>85 g</t>
         </is>
       </c>
       <c r="E45" s="133" t="inlineStr">
@@ -3907,7 +3907,7 @@
       </c>
       <c r="F45" s="133" t="inlineStr">
         <is>
-          <t>Mix Semințe de Floarea Soarelui și Dovleac 150g; Semințe crude de Dovleac 150g; Arahide crude 150g</t>
+          <t>Alune de pădure 85g</t>
         </is>
       </c>
       <c r="G45" s="132" t="n"/>
@@ -3937,22 +3937,22 @@
       </c>
       <c r="C46" s="133" t="inlineStr">
         <is>
-          <t>Punga 140 g</t>
+          <t>Rasnita 200 g (recipient + mecanism de macinare)</t>
         </is>
       </c>
       <c r="D46" s="133" t="inlineStr">
         <is>
-          <t>140 g</t>
+          <t>200 g</t>
         </is>
       </c>
       <c r="E46" s="133" t="inlineStr">
         <is>
-          <t>Transparenta + eticheta (din poza)</t>
+          <t>Transparent (recipient), negru (rasnita), din poza</t>
         </is>
       </c>
       <c r="F46" s="133" t="inlineStr">
         <is>
-          <t>Migdale crude 140 g</t>
+          <t>Sare roz de Himalaya Neiodată Râșniță 200g</t>
         </is>
       </c>
       <c r="G46" s="132" t="n"/>
@@ -3977,341 +3977,97 @@
       <c r="M46" s="138" t="n"/>
     </row>
     <row r="47" s="128">
-      <c r="B47" s="132" t="n">
-        <v>41</v>
-      </c>
-      <c r="C47" s="133" t="inlineStr">
-        <is>
-          <t>Punga 130 g</t>
-        </is>
-      </c>
-      <c r="D47" s="133" t="inlineStr">
-        <is>
-          <t>130 g</t>
-        </is>
-      </c>
-      <c r="E47" s="133" t="inlineStr">
-        <is>
-          <t>Transparenta + eticheta (din poza)</t>
-        </is>
-      </c>
-      <c r="F47" s="133" t="inlineStr">
-        <is>
-          <t>Semințe de In 130g; Omega Mix 130g; Stafide brune 130g; Mix Caju și Migdale 130g; Mix Fructe uscate și Nuci 130g; Fistic crud 130g</t>
-        </is>
-      </c>
+      <c r="B47" s="132" t="n"/>
+      <c r="C47" s="132" t="n"/>
+      <c r="D47" s="132" t="n"/>
+      <c r="E47" s="132" t="n"/>
+      <c r="F47" s="132" t="n"/>
       <c r="G47" s="132" t="n"/>
-      <c r="H47" s="134">
-        <f>IFERROR(INDIRECT("'"&amp;G47&amp;"'!E26"),"")</f>
-        <v/>
-      </c>
-      <c r="I47" s="135">
-        <f>IFERROR(INDIRECT("'"&amp;G47&amp;"'!E27"),"")</f>
-        <v/>
-      </c>
-      <c r="J47" s="136">
-        <f>IFERROR(INDIRECT("'"&amp;G47&amp;"'!E28"),"")</f>
-        <v/>
-      </c>
-      <c r="K47" s="137" t="n"/>
-      <c r="L47" s="137" t="inlineStr">
-        <is>
-          <t>In curs</t>
-        </is>
-      </c>
-      <c r="M47" s="138" t="n"/>
+      <c r="H47" s="132" t="n"/>
+      <c r="I47" s="132" t="n"/>
+      <c r="J47" s="132" t="n"/>
+      <c r="K47" s="132" t="n"/>
+      <c r="L47" s="132" t="n"/>
+      <c r="M47" s="132" t="n"/>
     </row>
     <row r="48" s="128">
-      <c r="B48" s="132" t="n">
-        <v>42</v>
-      </c>
-      <c r="C48" s="133" t="inlineStr">
-        <is>
-          <t>Punga 110 g</t>
-        </is>
-      </c>
-      <c r="D48" s="133" t="inlineStr">
-        <is>
-          <t>110 g</t>
-        </is>
-      </c>
-      <c r="E48" s="133" t="inlineStr">
-        <is>
-          <t>Transparenta + eticheta (din poza)</t>
-        </is>
-      </c>
-      <c r="F48" s="133" t="inlineStr">
-        <is>
-          <t>Caju crud 110g; Merișor 110g; Vitamin Mix Merișor și Goji 110g</t>
-        </is>
-      </c>
+      <c r="B48" s="132" t="n"/>
+      <c r="C48" s="132" t="n"/>
+      <c r="D48" s="132" t="n"/>
+      <c r="E48" s="132" t="n"/>
+      <c r="F48" s="132" t="n"/>
       <c r="G48" s="132" t="n"/>
-      <c r="H48" s="134">
-        <f>IFERROR(INDIRECT("'"&amp;G48&amp;"'!E26"),"")</f>
-        <v/>
-      </c>
-      <c r="I48" s="135">
-        <f>IFERROR(INDIRECT("'"&amp;G48&amp;"'!E27"),"")</f>
-        <v/>
-      </c>
-      <c r="J48" s="136">
-        <f>IFERROR(INDIRECT("'"&amp;G48&amp;"'!E28"),"")</f>
-        <v/>
-      </c>
-      <c r="K48" s="137" t="n"/>
-      <c r="L48" s="137" t="inlineStr">
-        <is>
-          <t>In curs</t>
-        </is>
-      </c>
-      <c r="M48" s="138" t="n"/>
-    </row>
-    <row r="49" s="128">
-      <c r="B49" s="132" t="n">
-        <v>43</v>
-      </c>
-      <c r="C49" s="133" t="inlineStr">
-        <is>
-          <t>Punga 100 g</t>
-        </is>
-      </c>
-      <c r="D49" s="133" t="inlineStr">
-        <is>
-          <t>100 g</t>
-        </is>
-      </c>
-      <c r="E49" s="133" t="inlineStr">
-        <is>
-          <t>Transparenta + eticheta (din poza)</t>
-        </is>
-      </c>
-      <c r="F49" s="133" t="inlineStr">
-        <is>
-          <t>Semințe de Chia 100g; Semințe de Susan 100g; Goji 100g</t>
-        </is>
-      </c>
-      <c r="G49" s="132" t="n"/>
-      <c r="H49" s="134">
-        <f>IFERROR(INDIRECT("'"&amp;G49&amp;"'!E26"),"")</f>
-        <v/>
-      </c>
-      <c r="I49" s="135">
-        <f>IFERROR(INDIRECT("'"&amp;G49&amp;"'!E27"),"")</f>
-        <v/>
-      </c>
-      <c r="J49" s="136">
-        <f>IFERROR(INDIRECT("'"&amp;G49&amp;"'!E28"),"")</f>
-        <v/>
-      </c>
-      <c r="K49" s="137" t="n"/>
-      <c r="L49" s="137" t="inlineStr">
-        <is>
-          <t>In curs</t>
-        </is>
-      </c>
-      <c r="M49" s="138" t="n"/>
-    </row>
-    <row r="50" s="128">
-      <c r="B50" s="132" t="n">
-        <v>44</v>
-      </c>
-      <c r="C50" s="133" t="inlineStr">
-        <is>
-          <t>Punga 85 g</t>
-        </is>
-      </c>
-      <c r="D50" s="133" t="inlineStr">
-        <is>
-          <t>85 g</t>
-        </is>
-      </c>
-      <c r="E50" s="133" t="inlineStr">
-        <is>
-          <t>Transparenta + eticheta (din poza)</t>
-        </is>
-      </c>
-      <c r="F50" s="133" t="inlineStr">
-        <is>
-          <t>Alune de pădure 85g</t>
-        </is>
-      </c>
-      <c r="G50" s="132" t="n"/>
-      <c r="H50" s="134">
-        <f>IFERROR(INDIRECT("'"&amp;G50&amp;"'!E26"),"")</f>
-        <v/>
-      </c>
-      <c r="I50" s="135">
-        <f>IFERROR(INDIRECT("'"&amp;G50&amp;"'!E27"),"")</f>
-        <v/>
-      </c>
-      <c r="J50" s="136">
-        <f>IFERROR(INDIRECT("'"&amp;G50&amp;"'!E28"),"")</f>
-        <v/>
-      </c>
-      <c r="K50" s="137" t="n"/>
-      <c r="L50" s="137" t="inlineStr">
-        <is>
-          <t>In curs</t>
-        </is>
-      </c>
-      <c r="M50" s="138" t="n"/>
-    </row>
-    <row r="51" s="128">
-      <c r="B51" s="132" t="n">
-        <v>45</v>
-      </c>
-      <c r="C51" s="133" t="inlineStr">
-        <is>
-          <t>Punga ceai 35 g</t>
-        </is>
-      </c>
-      <c r="D51" s="133" t="inlineStr">
-        <is>
-          <t>35 g</t>
-        </is>
-      </c>
-      <c r="E51" s="133" t="inlineStr">
-        <is>
-          <t>De confirmat</t>
-        </is>
-      </c>
-      <c r="F51" s="133" t="inlineStr">
-        <is>
-          <t>Ceai Rooibos cu vanilie 35g; Ceai Fructe de pădure cu scorțișoară 35g</t>
-        </is>
-      </c>
-      <c r="G51" s="132" t="n"/>
-      <c r="H51" s="134">
-        <f>IFERROR(INDIRECT("'"&amp;G51&amp;"'!E26"),"")</f>
-        <v/>
-      </c>
-      <c r="I51" s="135">
-        <f>IFERROR(INDIRECT("'"&amp;G51&amp;"'!E27"),"")</f>
-        <v/>
-      </c>
-      <c r="J51" s="136">
-        <f>IFERROR(INDIRECT("'"&amp;G51&amp;"'!E28"),"")</f>
-        <v/>
-      </c>
-      <c r="K51" s="137" t="n"/>
-      <c r="L51" s="137" t="inlineStr">
-        <is>
-          <t>In curs</t>
-        </is>
-      </c>
-      <c r="M51" s="138" t="n"/>
-    </row>
-    <row r="52" s="128">
-      <c r="B52" s="132" t="n">
-        <v>46</v>
-      </c>
-      <c r="C52" s="133" t="inlineStr">
-        <is>
-          <t>Rasnita 200 g (recipient + mecanism de macinare)</t>
-        </is>
-      </c>
-      <c r="D52" s="133" t="inlineStr">
-        <is>
-          <t>200 g</t>
-        </is>
-      </c>
-      <c r="E52" s="133" t="inlineStr">
-        <is>
-          <t>Transparent (recipient), negru (rasnita), din poza</t>
-        </is>
-      </c>
-      <c r="F52" s="133" t="inlineStr">
-        <is>
-          <t>Sare roz de Himalaya Neiodată Râșniță 200g</t>
-        </is>
-      </c>
-      <c r="G52" s="132" t="n"/>
-      <c r="H52" s="134">
-        <f>IFERROR(INDIRECT("'"&amp;G52&amp;"'!E26"),"")</f>
-        <v/>
-      </c>
-      <c r="I52" s="135">
-        <f>IFERROR(INDIRECT("'"&amp;G52&amp;"'!E27"),"")</f>
-        <v/>
-      </c>
-      <c r="J52" s="136">
-        <f>IFERROR(INDIRECT("'"&amp;G52&amp;"'!E28"),"")</f>
-        <v/>
-      </c>
-      <c r="K52" s="137" t="n"/>
-      <c r="L52" s="137" t="inlineStr">
-        <is>
-          <t>In curs</t>
-        </is>
-      </c>
-      <c r="M52" s="138" t="n"/>
-    </row>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55" ht="19.95" customHeight="1" s="128">
-      <c r="C55" s="76" t="inlineStr">
+      <c r="H48" s="132" t="n"/>
+      <c r="I48" s="132" t="n"/>
+      <c r="J48" s="132" t="n"/>
+      <c r="K48" s="132" t="n"/>
+      <c r="L48" s="132" t="n"/>
+      <c r="M48" s="132" t="n"/>
+    </row>
+    <row r="49" ht="19.95" customHeight="1" s="128">
+      <c r="C49" s="76" t="inlineStr">
         <is>
           <t>Rezumat (automat)</t>
         </is>
       </c>
-      <c r="D55" s="73" t="inlineStr">
+      <c r="D49" s="73" t="inlineStr">
         <is>
           <t>Nr. unitati</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="19.95" customHeight="1" s="128">
-      <c r="C56" s="74" t="inlineStr">
+    <row r="50" ht="19.95" customHeight="1" s="128">
+      <c r="C50" s="74" t="inlineStr">
         <is>
           <t>Unitati analizate</t>
         </is>
       </c>
-      <c r="D56" s="75">
-        <f>COUNTIF(G7:G52,"?*")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57" ht="19.95" customHeight="1" s="128">
-      <c r="C57" s="74" t="inlineStr">
+      <c r="D50" s="75">
+        <f>COUNTIF(G7:G46,"?*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="19.95" customHeight="1" s="128">
+      <c r="C51" s="74" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D57" s="75">
-        <f>COUNTIF($J$7:$J$52,C57)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58" ht="19.95" customHeight="1" s="128">
-      <c r="C58" s="74" t="inlineStr">
+      <c r="D51" s="75">
+        <f>COUNTIF($J$7:$J$46,C51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="19.95" customHeight="1" s="128">
+      <c r="C52" s="74" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="D58" s="75">
-        <f>COUNTIF($J$7:$J$52,C58)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59" ht="19.95" customHeight="1" s="128">
-      <c r="C59" s="74" t="inlineStr">
+      <c r="D52" s="75">
+        <f>COUNTIF($J$7:$J$46,C52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" ht="19.95" customHeight="1" s="128">
+      <c r="C53" s="74" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="D59" s="75">
-        <f>COUNTIF($J$7:$J$52,C59)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" ht="19.95" customHeight="1" s="128">
-      <c r="C60" s="74" t="inlineStr">
+      <c r="D53" s="75">
+        <f>COUNTIF($J$7:$J$46,C53)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" ht="19.95" customHeight="1" s="128">
+      <c r="C54" s="74" t="inlineStr">
         <is>
           <t>Sub 70% - nereciclabil</t>
         </is>
       </c>
-      <c r="D60" s="75">
-        <f>COUNTIF($J$7:$J$52,C60)</f>
+      <c r="D54" s="75">
+        <f>COUNTIF($J$7:$J$46,C54)</f>
         <v/>
       </c>
     </row>
@@ -4320,12 +4076,12 @@
     <mergeCell ref="B4:K4"/>
     <mergeCell ref="B2:K2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G7:G52">
+  <conditionalFormatting sqref="G7:G46">
     <cfRule type="expression" priority="4" dxfId="3">
       <formula>AND($G7&lt;&gt;"",$H7="")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J7:J52">
+  <conditionalFormatting sqref="J7:J46">
     <cfRule type="expression" priority="1" dxfId="2">
       <formula>OR($J7="A",$J7="B")</formula>
     </cfRule>
@@ -4337,10 +4093,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="K7:K52" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Prioritate" error="Alegeti: Mare, Medie sau Mica." type="list">
+    <dataValidation sqref="K7:K46" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Prioritate" error="Alegeti: Mare, Medie sau Mica." type="list">
       <formula1>"Mare,Medie,Mica"</formula1>
     </dataValidation>
-    <dataValidation sqref="L7:L52" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Stadiu analiza" error="Valoarea nu este in lista. Puteti continua daca este intentionat." type="list" errorStyle="information">
+    <dataValidation sqref="L7:L46" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Stadiu analiza" error="Valoarea nu este in lista. Puteti continua daca este intentionat." type="list" errorStyle="information">
       <formula1>"Identificata,In completare,Completa,Oferta trimisa"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>